<commit_message>
Refresh sample-report/ with citation fixes
Regenerated after fixing 15 evidence entries that were missing their
inline Source citation.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-report/stakeholder-review-all.xlsx
+++ b/sample-report/stakeholder-review-all.xlsx
@@ -3235,7 +3235,19 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Confirmed absent after independent gap-check: no citable feature found; searches for InsightAppSec plus partner/open-banking/third-party-risk terms returned only generic industry TPRM content unrelated to Rapid7.</t>
+          <r>
+            <t xml:space="preserve">Confirmed absent after independent gap-check: no citable feature found; searches for InsightAppSec plus partner/open-banking/third-party-risk terms returned only generic industry TPRM content unrelated to Rapid7. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>rapid7.com/products/insightappsec</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (no partner-API-specific feature found there or elsewhere)</t>
+          </r>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -4217,12 +4229,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4594,7 +4607,16 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Only a 'Discovery scan' vs. 'Vulnerability scan' mode distinction was found; no explicit passive-mode/rate-limiting documentation located for WAS specifically -- a genuine research gap relative to other vendors scored so far.</t>
+          <r>
+            <t xml:space="preserve">Only a 'Discovery scan' vs. 'Vulnerability scan' mode distinction was found; no explicit passive-mode/rate-limiting documentation located for WAS specifically -- a genuine research gap relative to other vendors scored so far. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>cdn2.qualys.com/docs/qualys-was-getting-started-guide.pdf</t>
+          </r>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
@@ -4886,7 +4908,7 @@
             <t>ASP.NET</t>
           </r>
           <r>
-            <t xml:space="preserve"> WebForms/JSP/mainframe-gateway-specific claims found for WAS.</t>
+            <t xml:space="preserve"> WebForms/JSP/mainframe-gateway-specific claims found for WAS. Source: qualys.com/apps/web-app-scanning</t>
           </r>
         </is>
       </c>
@@ -4949,7 +4971,16 @@
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>Confirmed weak after independent gap-check: 'Form Training' and Selenium/Browser-Recorder scripts enable crawling through multi-step workflows but no authorization-state-aware business-logic testing capability was found (nothing analogous to a privilege-escalation-diff test). A source explicitly states 'Standard DAST tools like Qualys WAS cannot validate business logic,' and this stands unrebutted.</t>
+          <r>
+            <t xml:space="preserve">Confirmed weak after independent gap-check: 'Form Training' and Selenium/Browser-Recorder scripts enable crawling through multi-step workflows but no authorization-state-aware business-logic testing capability was found (nothing analogous to a privilege-escalation-diff test). A source explicitly states 'Standard DAST tools like Qualys WAS cannot validate business logic,' and this stands unrebutted. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>getautonoma.com/blog/dast-tools</t>
+          </r>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
@@ -5233,7 +5264,16 @@
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>No independent benchmark or user-review data found specifically quantifying WAS's false-positive rate in either direction.</t>
+          <r>
+            <t xml:space="preserve">No independent benchmark or user-review data found specifically quantifying WAS's false-positive rate in either direction; the vendor's own product page makes no specific FP-rate claim either. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>qualys.com/apps/web-app-scanning</t>
+          </r>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr">
@@ -5295,7 +5335,19 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>TruRisk-based prioritization implied at the platform level; no WAS-specific instance-tailored remediation-guidance citation found distinct from generic vulnerability descriptions.</t>
+          <r>
+            <t xml:space="preserve">TruRisk-based prioritization implied at the platform level; no WAS-specific instance-tailored remediation-guidance citation found distinct from generic vulnerability descriptions. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>docs.qualys.com/en/vmdr/latest/trurisk/truRisk_report.htm</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (platform-wide, not WAS-specific)</t>
+          </r>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
@@ -5357,7 +5409,16 @@
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>Confirmed weak after independent gap-check: no cross-scan learning or automated proof-of-concept replay found beyond manual ignore/exception marking and TruRisk's risk-prioritization scoring.</t>
+          <r>
+            <t xml:space="preserve">Confirmed weak after independent gap-check: no cross-scan learning or automated proof-of-concept replay found beyond manual ignore/exception marking and TruRisk's risk-prioritization scoring. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>docs.qualys.com/en/was/latest/knowledgebase/ignore_vulnerability.htm</t>
+          </r>
         </is>
       </c>
       <c r="F17" s="16" t="inlineStr">
@@ -6082,7 +6143,16 @@
       </c>
       <c r="E27" s="18" t="inlineStr">
         <is>
-          <t>Vendor claims ML-optimized scan patterns reduce scan time by up to 80% on large applications -- self-reported, but a specific number.</t>
+          <r>
+            <t xml:space="preserve">Vendor claims ML-optimized scan patterns reduce scan time by up to 80% on large applications -- self-reported, but a specific number. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>qualys.com/apps/web-app-scanning</t>
+          </r>
         </is>
       </c>
       <c r="F27" s="16" t="inlineStr">
@@ -6366,7 +6436,16 @@
       </c>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>Confirmed absent after independent gap-check: no IDE plugin (VS Code, IntelliJ, Eclipse) or pre-commit tool found anywhere for WAS; only the CI/CD Jenkins plugin exists, which is pipeline integration, not local/IDE tooling.</t>
+          <r>
+            <t xml:space="preserve">Confirmed absent after independent gap-check: no IDE plugin (VS Code, IntelliJ, Eclipse) or pre-commit tool found anywhere for WAS; only the CI/CD Jenkins plugin exists, which is pipeline integration, not local/IDE tooling. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>plugins.jenkins.io/qualys-was</t>
+          </r>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
@@ -6499,7 +6578,16 @@
       </c>
       <c r="E33" s="18" t="inlineStr">
         <is>
-          <t>Confirmed absent after independent gap-check: Qualys's partner/vendor-asset content is under CSAM ('Import Third-Party Assets API') for general asset inventory, not a WAS-specific partner-API-differentiated scanning or risk-program-formatted output.</t>
+          <r>
+            <t xml:space="preserve">Confirmed absent after independent gap-check: Qualys's partner/vendor-asset content is under CSAM ('Import Third-Party Assets API') for general asset inventory, not a WAS-specific partner-API-differentiated scanning or risk-program-formatted output. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>qualys.com/faqs-resources-attack-surface-management</t>
+          </r>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
@@ -6635,7 +6723,16 @@
       </c>
       <c r="E35" s="18" t="inlineStr">
         <is>
-          <t>Confirmed absent for WAS after independent gap-check: Qualys does have an 'Auto-Remediation' feature, but it is scoped to Policy Compliance (CAR scripts fixing infrastructure misconfigurations) and VMDR patch/ticket remediation -- not WAS, and not code-fix/PR generation.</t>
+          <r>
+            <t xml:space="preserve">Confirmed absent for WAS after independent gap-check: Qualys does have an 'Auto-Remediation' feature, but it is scoped to Policy Compliance (CAR scripts fixing infrastructure misconfigurations) and VMDR patch/ticket remediation -- not WAS, and not code-fix/PR generation. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>blog.qualys.com/product-tech/2023/04/03/augment-security-asset-tagging-with-custom-assessment-and-remediation-car</t>
+          </r>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
@@ -7235,28 +7332,37 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14367,7 +14473,16 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>OWASP Top 10 and OWASP API Security Top 10 mapping confirmed; no explicit PCI-DSS/GLBA/SOX/FFIEC/NYDFS regulatory-framework mapping found in DAST-specific documentation, though the platform broadly targets enterprise/regulated customers.</t>
+          <r>
+            <t xml:space="preserve">OWASP Top 10 and OWASP API Security Top 10 mapping confirmed; no explicit PCI-DSS/GLBA/SOX/FFIEC/NYDFS regulatory-framework mapping found in DAST-specific documentation, though the platform broadly targets enterprise/regulated customers. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>checkmarx.com/learn/integrating-dast-and-sast-into-devsecops-for-continuous-api-security</t>
+          </r>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
@@ -14429,7 +14544,16 @@
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>Proof-based scanning validates findings before flagging, and SAST-DAST correlation is cited to reduce noise -- but the vendor's own '89% noise reduction' figure applies to platform-wide ASPM correlation across all scanners, not a DAST-isolated false-positive rate, so it's cited here with that caveat rather than at face value.</t>
+          <r>
+            <t xml:space="preserve">Proof-based scanning validates findings before flagging, and SAST-DAST correlation is cited to reduce noise -- but the vendor's own '89% noise reduction' figure applies to platform-wide ASPM correlation across all scanners, not a DAST-isolated false-positive rate, so it's cited here with that caveat rather than at face value. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>checkmarx.com/blog/checkmarx-dast-for-the-ai-coding-era</t>
+          </r>
         </is>
       </c>
       <c r="F13" s="16" t="inlineStr">
@@ -16609,29 +16733,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18403,7 +18529,16 @@
       </c>
       <c r="E25" s="18" t="inlineStr">
         <is>
-          <t>AppScan on Cloud aggregates and correlates DAST, SAST, and IAST findings to provide proof of exploitability, prioritizing the most critical confirmed issues. Source: general platform documentation</t>
+          <r>
+            <t xml:space="preserve">AppScan on Cloud aggregates and correlates DAST, SAST, and IAST findings to provide proof of exploitability, prioritizing the most critical confirmed issues. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>hcl-software.com/appscan</t>
+          </r>
         </is>
       </c>
       <c r="F25" s="16" t="inlineStr">
@@ -18903,7 +19038,16 @@
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>API-level discovery/inventory confirmed via the Salt Security partnership; not confirmed at the rubric's top tier of scanning public IP ranges/domains for rogue unmapped apps.</t>
+          <r>
+            <t xml:space="preserve">API-level discovery/inventory confirmed via the Salt Security partnership; not confirmed at the rubric's top tier of scanning public IP ranges/domains for rogue unmapped apps. Source: </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="000563C1"/>
+              <u val="single"/>
+            </rPr>
+            <t>hcl-software.com/appscan/products/api-security</t>
+          </r>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
@@ -19742,16 +19886,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>